<commit_message>
rewrited nbc. py. Counted apriori_P in new nbc.py
</commit_message>
<xml_diff>
--- a/GrokLM/2.NBC/dataset.xlsx
+++ b/GrokLM/2.NBC/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\py\GrokLM\2.NBC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11CBF1C7-FEEE-467F-B049-64272A2325C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580F7D8C-3E47-4E65-8754-131E8B126C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
   <si>
     <t>№</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Патруль</t>
   </si>
   <si>
-    <t>Свой</t>
-  </si>
-  <si>
     <t>Мультикам</t>
   </si>
   <si>
@@ -63,9 +60,6 @@
     <t>G36</t>
   </si>
   <si>
-    <t>Враг</t>
-  </si>
-  <si>
     <t>M4A4</t>
   </si>
   <si>
@@ -79,6 +73,18 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>Первый</t>
+  </si>
+  <si>
+    <t>Второй</t>
+  </si>
+  <si>
+    <t>Третий</t>
+  </si>
+  <si>
+    <t>Четвертый</t>
   </si>
 </sst>
 </file>
@@ -413,14 +419,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
     <col min="4" max="4" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -437,7 +443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -451,10 +457,10 @@
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -465,18 +471,18 @@
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
@@ -485,78 +491,79 @@
         <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>11</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -564,36 +571,53 @@
         <v>5</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reviewed nbc.py; started linreg
</commit_message>
<xml_diff>
--- a/GrokLM/2.NBC/dataset.xlsx
+++ b/GrokLM/2.NBC/dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\py\GrokLM\2.NBC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{580F7D8C-3E47-4E65-8754-131E8B126C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08DD7F3F-4C48-42F3-B9F3-82FB35249FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2955" yWindow="1890" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="18">
   <si>
     <t>№</t>
   </si>
@@ -75,23 +75,17 @@
     <t>?</t>
   </si>
   <si>
-    <t>Первый</t>
-  </si>
-  <si>
-    <t>Второй</t>
-  </si>
-  <si>
-    <t>Третий</t>
-  </si>
-  <si>
-    <t>Четвертый</t>
+    <t>Свой</t>
+  </si>
+  <si>
+    <t>Враг</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,13 +101,39 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -125,10 +145,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -139,9 +161,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Плохой" xfId="2" builtinId="27"/>
+    <cellStyle name="Хороший" xfId="1" builtinId="26"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -419,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -444,185 +474,169 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>16</v>
       </c>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="B7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="B8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="D9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="C11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A10:E10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>